<commit_message>
Switch ENISA line: Jóvenes Emprendedores → Emprendedores (founder 57 yo)
Global changes due to founder birthday 1968 (57 yo, exceeds Jóvenes 40 limit):
- Plan de Empresa v2.2: all 13 numbers recalc for new ENISA terms
  (TIN 4.25→4.75%, carencia 12→24 months, plazo 84→96 months)
- Pitch deck slide 11: new ENISA terms
- CV founder v1: fully filled from user input (DOB 21/04/1968,
  Univ. Petrozavodsk Economics 1999, Machine-building Technikum,
  SignalWaves Auto = cars import DE→ES Barcelona garage,
  PsychAuto ~1000 tests, Construction 2000-2020, EN B1, ES A1,
  Spain resident since 2024)
- Financial model v2.2: EBITDA unchanged, IS/Neto adjusted
  for new interest schedule (Y1-Y2 interest-only at 297€/mo)

Outcome: Y3 caja 1.78M€ (vs 1.77M€), Y2 Neto 445k€ (vs 436k€) —
slightly better due to extended grace period.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/modelo-financiero-forged-wheels-v2.xlsx
+++ b/docs/modelo-financiero-forged-wheels-v2.xlsx
@@ -871,13 +871,13 @@
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>3192</v>
+        <v>3564</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>14184</v>
+        <v>3564</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>14184</v>
+        <v>14388</v>
       </c>
     </row>
     <row r="23">
@@ -887,13 +887,13 @@
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>-46383</v>
+        <v>-46755</v>
       </c>
       <c r="C23" s="7" t="n">
-        <v>513140</v>
+        <v>523760</v>
       </c>
       <c r="D23" s="7" t="n">
-        <v>2191546</v>
+        <v>2191342</v>
       </c>
     </row>
     <row r="24">
@@ -906,10 +906,10 @@
         <v>0</v>
       </c>
       <c r="C24" s="7" t="n">
-        <v>76971</v>
+        <v>78564</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>547886.5</v>
+        <v>547835.5</v>
       </c>
     </row>
     <row r="25">
@@ -919,13 +919,13 @@
         </is>
       </c>
       <c r="B25" s="9" t="n">
-        <v>-46383</v>
+        <v>-46755</v>
       </c>
       <c r="C25" s="9" t="n">
-        <v>436168</v>
+        <v>445196</v>
       </c>
       <c r="D25" s="9" t="n">
-        <v>1643658</v>
+        <v>1643506</v>
       </c>
     </row>
     <row r="26">
@@ -935,13 +935,13 @@
         </is>
       </c>
       <c r="B26" s="10" t="n">
-        <v>-21.47361111111111</v>
+        <v>-21.64583333333333</v>
       </c>
       <c r="C26" s="10" t="n">
-        <v>25.07289031961371</v>
+        <v>25.59186019774661</v>
       </c>
       <c r="D26" s="10" t="n">
-        <v>30.45164517563361</v>
+        <v>30.44882910923373</v>
       </c>
     </row>
     <row r="27">
@@ -951,13 +951,13 @@
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>52233</v>
+        <v>51861</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>452282</v>
+        <v>460938</v>
       </c>
       <c r="D27" s="7" t="n">
-        <v>1775677</v>
+        <v>1784181</v>
       </c>
     </row>
     <row r="31">
@@ -3738,121 +3738,121 @@
         </is>
       </c>
       <c r="B26" s="20" t="n">
-        <v>266</v>
+        <v>297</v>
       </c>
       <c r="C26" s="20" t="n">
-        <v>266</v>
+        <v>297</v>
       </c>
       <c r="D26" s="20" t="n">
-        <v>266</v>
+        <v>297</v>
       </c>
       <c r="E26" s="20" t="n">
-        <v>266</v>
+        <v>297</v>
       </c>
       <c r="F26" s="20" t="n">
-        <v>266</v>
+        <v>297</v>
       </c>
       <c r="G26" s="20" t="n">
-        <v>266</v>
+        <v>297</v>
       </c>
       <c r="H26" s="20" t="n">
-        <v>266</v>
+        <v>297</v>
       </c>
       <c r="I26" s="20" t="n">
-        <v>266</v>
+        <v>297</v>
       </c>
       <c r="J26" s="20" t="n">
-        <v>266</v>
+        <v>297</v>
       </c>
       <c r="K26" s="20" t="n">
-        <v>266</v>
+        <v>297</v>
       </c>
       <c r="L26" s="20" t="n">
-        <v>266</v>
+        <v>297</v>
       </c>
       <c r="M26" s="20" t="n">
-        <v>266</v>
+        <v>297</v>
       </c>
       <c r="N26" s="20" t="n">
-        <v>1182</v>
+        <v>297</v>
       </c>
       <c r="O26" s="20" t="n">
-        <v>1182</v>
+        <v>297</v>
       </c>
       <c r="P26" s="20" t="n">
-        <v>1182</v>
+        <v>297</v>
       </c>
       <c r="Q26" s="20" t="n">
-        <v>1182</v>
+        <v>297</v>
       </c>
       <c r="R26" s="20" t="n">
-        <v>1182</v>
+        <v>297</v>
       </c>
       <c r="S26" s="20" t="n">
-        <v>1182</v>
+        <v>297</v>
       </c>
       <c r="T26" s="20" t="n">
-        <v>1182</v>
+        <v>297</v>
       </c>
       <c r="U26" s="20" t="n">
-        <v>1182</v>
+        <v>297</v>
       </c>
       <c r="V26" s="20" t="n">
-        <v>1182</v>
+        <v>297</v>
       </c>
       <c r="W26" s="20" t="n">
-        <v>1182</v>
+        <v>297</v>
       </c>
       <c r="X26" s="20" t="n">
-        <v>1182</v>
+        <v>297</v>
       </c>
       <c r="Y26" s="20" t="n">
-        <v>1182</v>
+        <v>297</v>
       </c>
       <c r="Z26" s="20" t="n">
-        <v>1182</v>
+        <v>1199</v>
       </c>
       <c r="AA26" s="20" t="n">
-        <v>1182</v>
+        <v>1199</v>
       </c>
       <c r="AB26" s="20" t="n">
-        <v>1182</v>
+        <v>1199</v>
       </c>
       <c r="AC26" s="20" t="n">
-        <v>1182</v>
+        <v>1199</v>
       </c>
       <c r="AD26" s="20" t="n">
-        <v>1182</v>
+        <v>1199</v>
       </c>
       <c r="AE26" s="20" t="n">
-        <v>1182</v>
+        <v>1199</v>
       </c>
       <c r="AF26" s="20" t="n">
-        <v>1182</v>
+        <v>1199</v>
       </c>
       <c r="AG26" s="20" t="n">
-        <v>1182</v>
+        <v>1199</v>
       </c>
       <c r="AH26" s="20" t="n">
-        <v>1182</v>
+        <v>1199</v>
       </c>
       <c r="AI26" s="20" t="n">
-        <v>1182</v>
+        <v>1199</v>
       </c>
       <c r="AJ26" s="20" t="n">
-        <v>1182</v>
+        <v>1199</v>
       </c>
       <c r="AK26" s="20" t="n">
-        <v>1182</v>
+        <v>1199</v>
       </c>
       <c r="AL26" s="21" t="n">
-        <v>3192</v>
+        <v>3564</v>
       </c>
       <c r="AM26" s="21" t="n">
-        <v>14184</v>
+        <v>3564</v>
       </c>
       <c r="AN26" s="21" t="n">
-        <v>14184</v>
+        <v>14388</v>
       </c>
     </row>
     <row r="27">
@@ -3862,121 +3862,121 @@
         </is>
       </c>
       <c r="B27" s="18" t="n">
-        <v>-19091</v>
+        <v>-19122</v>
       </c>
       <c r="C27" s="18" t="n">
-        <v>-11146</v>
+        <v>-11177</v>
       </c>
       <c r="D27" s="18" t="n">
-        <v>-9576</v>
+        <v>-9607</v>
       </c>
       <c r="E27" s="18" t="n">
-        <v>-4634</v>
+        <v>-4665</v>
       </c>
       <c r="F27" s="18" t="n">
-        <v>-3424</v>
+        <v>-3455</v>
       </c>
       <c r="G27" s="18" t="n">
-        <v>-2215</v>
+        <v>-2246</v>
       </c>
       <c r="H27" s="18" t="n">
-        <v>-1600</v>
+        <v>-1631</v>
       </c>
       <c r="I27" s="18" t="n">
-        <v>-391</v>
+        <v>-422</v>
       </c>
       <c r="J27" s="18" t="n">
-        <v>214</v>
+        <v>183</v>
       </c>
       <c r="K27" s="18" t="n">
-        <v>819</v>
+        <v>788</v>
       </c>
       <c r="L27" s="18" t="n">
-        <v>2028</v>
+        <v>1997</v>
       </c>
       <c r="M27" s="18" t="n">
-        <v>2633</v>
+        <v>2602</v>
       </c>
       <c r="N27" s="18" t="n">
-        <v>23204</v>
+        <v>24089</v>
       </c>
       <c r="O27" s="18" t="n">
-        <v>27114</v>
+        <v>27999</v>
       </c>
       <c r="P27" s="18" t="n">
-        <v>30242</v>
+        <v>31127</v>
       </c>
       <c r="Q27" s="18" t="n">
-        <v>33370</v>
+        <v>34255</v>
       </c>
       <c r="R27" s="18" t="n">
-        <v>40408</v>
+        <v>41293</v>
       </c>
       <c r="S27" s="18" t="n">
-        <v>43536</v>
+        <v>44421</v>
       </c>
       <c r="T27" s="18" t="n">
-        <v>40684</v>
+        <v>41569</v>
       </c>
       <c r="U27" s="18" t="n">
-        <v>43812</v>
+        <v>44697</v>
       </c>
       <c r="V27" s="18" t="n">
-        <v>47722</v>
+        <v>48607</v>
       </c>
       <c r="W27" s="18" t="n">
-        <v>50850</v>
+        <v>51735</v>
       </c>
       <c r="X27" s="18" t="n">
-        <v>61016</v>
+        <v>61901</v>
       </c>
       <c r="Y27" s="18" t="n">
-        <v>71182</v>
+        <v>72067</v>
       </c>
       <c r="Z27" s="18" t="n">
-        <v>121240</v>
+        <v>121223</v>
       </c>
       <c r="AA27" s="18" t="n">
-        <v>131791</v>
+        <v>131774</v>
       </c>
       <c r="AB27" s="18" t="n">
-        <v>142342</v>
+        <v>142325</v>
       </c>
       <c r="AC27" s="18" t="n">
-        <v>153853</v>
+        <v>153836</v>
       </c>
       <c r="AD27" s="18" t="n">
-        <v>164404</v>
+        <v>164387</v>
       </c>
       <c r="AE27" s="18" t="n">
-        <v>174955</v>
+        <v>174938</v>
       </c>
       <c r="AF27" s="18" t="n">
-        <v>186466</v>
+        <v>186449</v>
       </c>
       <c r="AG27" s="18" t="n">
-        <v>197017</v>
+        <v>197000</v>
       </c>
       <c r="AH27" s="18" t="n">
-        <v>207568</v>
+        <v>207551</v>
       </c>
       <c r="AI27" s="18" t="n">
-        <v>219078</v>
+        <v>219061</v>
       </c>
       <c r="AJ27" s="18" t="n">
-        <v>229630</v>
+        <v>229613</v>
       </c>
       <c r="AK27" s="18" t="n">
-        <v>263202</v>
+        <v>263185</v>
       </c>
       <c r="AL27" s="19" t="n">
-        <v>-46383</v>
+        <v>-46755</v>
       </c>
       <c r="AM27" s="19" t="n">
-        <v>513140</v>
+        <v>523760</v>
       </c>
       <c r="AN27" s="19" t="n">
-        <v>2191546</v>
+        <v>2191342</v>
       </c>
     </row>
     <row r="28">
@@ -4028,7 +4028,7 @@
         <v>0</v>
       </c>
       <c r="P28" s="20" t="n">
-        <v>19243</v>
+        <v>19641</v>
       </c>
       <c r="Q28" s="20" t="n">
         <v>0</v>
@@ -4037,7 +4037,7 @@
         <v>0</v>
       </c>
       <c r="S28" s="20" t="n">
-        <v>19243</v>
+        <v>19641</v>
       </c>
       <c r="T28" s="20" t="n">
         <v>0</v>
@@ -4046,7 +4046,7 @@
         <v>0</v>
       </c>
       <c r="V28" s="20" t="n">
-        <v>19243</v>
+        <v>19641</v>
       </c>
       <c r="W28" s="20" t="n">
         <v>0</v>
@@ -4055,7 +4055,7 @@
         <v>0</v>
       </c>
       <c r="Y28" s="20" t="n">
-        <v>19243</v>
+        <v>19641</v>
       </c>
       <c r="Z28" s="20" t="n">
         <v>0</v>
@@ -4064,7 +4064,7 @@
         <v>0</v>
       </c>
       <c r="AB28" s="20" t="n">
-        <v>136972</v>
+        <v>136959</v>
       </c>
       <c r="AC28" s="20" t="n">
         <v>0</v>
@@ -4073,7 +4073,7 @@
         <v>0</v>
       </c>
       <c r="AE28" s="20" t="n">
-        <v>136972</v>
+        <v>136959</v>
       </c>
       <c r="AF28" s="20" t="n">
         <v>0</v>
@@ -4082,7 +4082,7 @@
         <v>0</v>
       </c>
       <c r="AH28" s="20" t="n">
-        <v>136972</v>
+        <v>136959</v>
       </c>
       <c r="AI28" s="20" t="n">
         <v>0</v>
@@ -4091,16 +4091,16 @@
         <v>0</v>
       </c>
       <c r="AK28" s="20" t="n">
-        <v>136972</v>
+        <v>136959</v>
       </c>
       <c r="AL28" s="21" t="n">
         <v>0</v>
       </c>
       <c r="AM28" s="21" t="n">
-        <v>76972</v>
+        <v>78564</v>
       </c>
       <c r="AN28" s="21" t="n">
-        <v>547888</v>
+        <v>547836</v>
       </c>
     </row>
     <row r="29">
@@ -4110,121 +4110,121 @@
         </is>
       </c>
       <c r="B29" s="22" t="n">
-        <v>-19091</v>
+        <v>-19122</v>
       </c>
       <c r="C29" s="22" t="n">
-        <v>-11146</v>
+        <v>-11177</v>
       </c>
       <c r="D29" s="22" t="n">
-        <v>-9576</v>
+        <v>-9607</v>
       </c>
       <c r="E29" s="22" t="n">
-        <v>-4634</v>
+        <v>-4665</v>
       </c>
       <c r="F29" s="22" t="n">
-        <v>-3424</v>
+        <v>-3455</v>
       </c>
       <c r="G29" s="22" t="n">
-        <v>-2215</v>
+        <v>-2246</v>
       </c>
       <c r="H29" s="22" t="n">
-        <v>-1600</v>
+        <v>-1631</v>
       </c>
       <c r="I29" s="22" t="n">
-        <v>-391</v>
+        <v>-422</v>
       </c>
       <c r="J29" s="22" t="n">
-        <v>214</v>
+        <v>183</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>819</v>
+        <v>788</v>
       </c>
       <c r="L29" s="22" t="n">
-        <v>2028</v>
+        <v>1997</v>
       </c>
       <c r="M29" s="22" t="n">
-        <v>2633</v>
+        <v>2602</v>
       </c>
       <c r="N29" s="22" t="n">
-        <v>23204</v>
+        <v>24089</v>
       </c>
       <c r="O29" s="22" t="n">
-        <v>27114</v>
+        <v>27999</v>
       </c>
       <c r="P29" s="22" t="n">
-        <v>10999</v>
+        <v>11486</v>
       </c>
       <c r="Q29" s="22" t="n">
-        <v>33370</v>
+        <v>34255</v>
       </c>
       <c r="R29" s="22" t="n">
-        <v>40408</v>
+        <v>41293</v>
       </c>
       <c r="S29" s="22" t="n">
-        <v>24293</v>
+        <v>24780</v>
       </c>
       <c r="T29" s="22" t="n">
-        <v>40684</v>
+        <v>41569</v>
       </c>
       <c r="U29" s="22" t="n">
-        <v>43812</v>
+        <v>44697</v>
       </c>
       <c r="V29" s="22" t="n">
-        <v>28479</v>
+        <v>28966</v>
       </c>
       <c r="W29" s="22" t="n">
-        <v>50850</v>
+        <v>51735</v>
       </c>
       <c r="X29" s="22" t="n">
-        <v>61016</v>
+        <v>61901</v>
       </c>
       <c r="Y29" s="22" t="n">
-        <v>51939</v>
+        <v>52426</v>
       </c>
       <c r="Z29" s="22" t="n">
-        <v>121240</v>
+        <v>121223</v>
       </c>
       <c r="AA29" s="22" t="n">
-        <v>131791</v>
+        <v>131774</v>
       </c>
       <c r="AB29" s="22" t="n">
-        <v>5370</v>
+        <v>5366</v>
       </c>
       <c r="AC29" s="22" t="n">
-        <v>153853</v>
+        <v>153836</v>
       </c>
       <c r="AD29" s="22" t="n">
-        <v>164404</v>
+        <v>164387</v>
       </c>
       <c r="AE29" s="22" t="n">
-        <v>37983</v>
+        <v>37979</v>
       </c>
       <c r="AF29" s="22" t="n">
-        <v>186466</v>
+        <v>186449</v>
       </c>
       <c r="AG29" s="22" t="n">
-        <v>197017</v>
+        <v>197000</v>
       </c>
       <c r="AH29" s="22" t="n">
-        <v>70596</v>
+        <v>70592</v>
       </c>
       <c r="AI29" s="22" t="n">
-        <v>219078</v>
+        <v>219061</v>
       </c>
       <c r="AJ29" s="22" t="n">
-        <v>229630</v>
+        <v>229613</v>
       </c>
       <c r="AK29" s="22" t="n">
-        <v>126230</v>
+        <v>126226</v>
       </c>
       <c r="AL29" s="19" t="n">
-        <v>-46383</v>
+        <v>-46755</v>
       </c>
       <c r="AM29" s="19" t="n">
-        <v>436168</v>
+        <v>445196</v>
       </c>
       <c r="AN29" s="19" t="n">
-        <v>1643658</v>
+        <v>1643506</v>
       </c>
     </row>
     <row r="30">
@@ -5631,7 +5631,7 @@
         <v>0</v>
       </c>
       <c r="P11" s="20" t="n">
-        <v>-19243</v>
+        <v>-19641</v>
       </c>
       <c r="Q11" s="20" t="n">
         <v>0</v>
@@ -5640,7 +5640,7 @@
         <v>0</v>
       </c>
       <c r="S11" s="20" t="n">
-        <v>-19243</v>
+        <v>-19641</v>
       </c>
       <c r="T11" s="20" t="n">
         <v>0</v>
@@ -5649,7 +5649,7 @@
         <v>0</v>
       </c>
       <c r="V11" s="20" t="n">
-        <v>-19243</v>
+        <v>-19641</v>
       </c>
       <c r="W11" s="20" t="n">
         <v>0</v>
@@ -5658,7 +5658,7 @@
         <v>0</v>
       </c>
       <c r="Y11" s="20" t="n">
-        <v>-19243</v>
+        <v>-19641</v>
       </c>
       <c r="Z11" s="20" t="n">
         <v>0</v>
@@ -5667,7 +5667,7 @@
         <v>0</v>
       </c>
       <c r="AB11" s="20" t="n">
-        <v>-136972</v>
+        <v>-136959</v>
       </c>
       <c r="AC11" s="20" t="n">
         <v>0</v>
@@ -5676,7 +5676,7 @@
         <v>0</v>
       </c>
       <c r="AE11" s="20" t="n">
-        <v>-136972</v>
+        <v>-136959</v>
       </c>
       <c r="AF11" s="20" t="n">
         <v>0</v>
@@ -5685,7 +5685,7 @@
         <v>0</v>
       </c>
       <c r="AH11" s="20" t="n">
-        <v>-136972</v>
+        <v>-136959</v>
       </c>
       <c r="AI11" s="20" t="n">
         <v>0</v>
@@ -5694,7 +5694,7 @@
         <v>0</v>
       </c>
       <c r="AK11" s="20" t="n">
-        <v>-136972</v>
+        <v>-136959</v>
       </c>
     </row>
     <row r="12">
@@ -5934,112 +5934,112 @@
         </is>
       </c>
       <c r="B14" s="20" t="n">
-        <v>-266</v>
+        <v>-297</v>
       </c>
       <c r="C14" s="20" t="n">
-        <v>-266</v>
+        <v>-297</v>
       </c>
       <c r="D14" s="20" t="n">
-        <v>-266</v>
+        <v>-297</v>
       </c>
       <c r="E14" s="20" t="n">
-        <v>-266</v>
+        <v>-297</v>
       </c>
       <c r="F14" s="20" t="n">
-        <v>-266</v>
+        <v>-297</v>
       </c>
       <c r="G14" s="20" t="n">
-        <v>-266</v>
+        <v>-297</v>
       </c>
       <c r="H14" s="20" t="n">
-        <v>-266</v>
+        <v>-297</v>
       </c>
       <c r="I14" s="20" t="n">
-        <v>-266</v>
+        <v>-297</v>
       </c>
       <c r="J14" s="20" t="n">
-        <v>-266</v>
+        <v>-297</v>
       </c>
       <c r="K14" s="20" t="n">
-        <v>-266</v>
+        <v>-297</v>
       </c>
       <c r="L14" s="20" t="n">
-        <v>-266</v>
+        <v>-297</v>
       </c>
       <c r="M14" s="20" t="n">
-        <v>-266</v>
+        <v>-297</v>
       </c>
       <c r="N14" s="20" t="n">
-        <v>-1182</v>
+        <v>-297</v>
       </c>
       <c r="O14" s="20" t="n">
-        <v>-1182</v>
+        <v>-297</v>
       </c>
       <c r="P14" s="20" t="n">
-        <v>-1182</v>
+        <v>-297</v>
       </c>
       <c r="Q14" s="20" t="n">
-        <v>-1182</v>
+        <v>-297</v>
       </c>
       <c r="R14" s="20" t="n">
-        <v>-1182</v>
+        <v>-297</v>
       </c>
       <c r="S14" s="20" t="n">
-        <v>-1182</v>
+        <v>-297</v>
       </c>
       <c r="T14" s="20" t="n">
-        <v>-1182</v>
+        <v>-297</v>
       </c>
       <c r="U14" s="20" t="n">
-        <v>-1182</v>
+        <v>-297</v>
       </c>
       <c r="V14" s="20" t="n">
-        <v>-1182</v>
+        <v>-297</v>
       </c>
       <c r="W14" s="20" t="n">
-        <v>-1182</v>
+        <v>-297</v>
       </c>
       <c r="X14" s="20" t="n">
-        <v>-1182</v>
+        <v>-297</v>
       </c>
       <c r="Y14" s="20" t="n">
-        <v>-1182</v>
+        <v>-297</v>
       </c>
       <c r="Z14" s="20" t="n">
-        <v>-1182</v>
+        <v>-1199</v>
       </c>
       <c r="AA14" s="20" t="n">
-        <v>-1182</v>
+        <v>-1199</v>
       </c>
       <c r="AB14" s="20" t="n">
-        <v>-1182</v>
+        <v>-1199</v>
       </c>
       <c r="AC14" s="20" t="n">
-        <v>-1182</v>
+        <v>-1199</v>
       </c>
       <c r="AD14" s="20" t="n">
-        <v>-1182</v>
+        <v>-1199</v>
       </c>
       <c r="AE14" s="20" t="n">
-        <v>-1182</v>
+        <v>-1199</v>
       </c>
       <c r="AF14" s="20" t="n">
-        <v>-1182</v>
+        <v>-1199</v>
       </c>
       <c r="AG14" s="20" t="n">
-        <v>-1182</v>
+        <v>-1199</v>
       </c>
       <c r="AH14" s="20" t="n">
-        <v>-1182</v>
+        <v>-1199</v>
       </c>
       <c r="AI14" s="20" t="n">
-        <v>-1182</v>
+        <v>-1199</v>
       </c>
       <c r="AJ14" s="20" t="n">
-        <v>-1182</v>
+        <v>-1199</v>
       </c>
       <c r="AK14" s="20" t="n">
-        <v>-1182</v>
+        <v>-1199</v>
       </c>
     </row>
     <row r="15">
@@ -6049,112 +6049,112 @@
         </is>
       </c>
       <c r="B15" s="19" t="n">
-        <v>56859</v>
+        <v>56828</v>
       </c>
       <c r="C15" s="19" t="n">
-        <v>-10196</v>
+        <v>-10227</v>
       </c>
       <c r="D15" s="19" t="n">
-        <v>-9873</v>
+        <v>-9904</v>
       </c>
       <c r="E15" s="19" t="n">
-        <v>-1342</v>
+        <v>-1373</v>
       </c>
       <c r="F15" s="19" t="n">
-        <v>-1082</v>
+        <v>-1113</v>
       </c>
       <c r="G15" s="19" t="n">
-        <v>-97</v>
+        <v>-128</v>
       </c>
       <c r="H15" s="19" t="n">
-        <v>1692</v>
+        <v>1661</v>
       </c>
       <c r="I15" s="19" t="n">
-        <v>1951</v>
+        <v>1920</v>
       </c>
       <c r="J15" s="19" t="n">
-        <v>-495</v>
+        <v>-526</v>
       </c>
       <c r="K15" s="19" t="n">
-        <v>2211</v>
+        <v>2180</v>
       </c>
       <c r="L15" s="19" t="n">
-        <v>4370</v>
+        <v>4339</v>
       </c>
       <c r="M15" s="19" t="n">
-        <v>235</v>
+        <v>204</v>
       </c>
       <c r="N15" s="19" t="n">
-        <v>47596</v>
+        <v>48481</v>
       </c>
       <c r="O15" s="19" t="n">
-        <v>32556</v>
+        <v>33441</v>
       </c>
       <c r="P15" s="19" t="n">
-        <v>-6556</v>
+        <v>-6069</v>
       </c>
       <c r="Q15" s="19" t="n">
-        <v>37812</v>
+        <v>38697</v>
       </c>
       <c r="R15" s="19" t="n">
-        <v>49850</v>
+        <v>50735</v>
       </c>
       <c r="S15" s="19" t="n">
-        <v>-1653</v>
+        <v>-1166</v>
       </c>
       <c r="T15" s="19" t="n">
-        <v>45126</v>
+        <v>46011</v>
       </c>
       <c r="U15" s="19" t="n">
-        <v>48254</v>
+        <v>49139</v>
       </c>
       <c r="V15" s="19" t="n">
-        <v>-1271</v>
+        <v>-784</v>
       </c>
       <c r="W15" s="19" t="n">
-        <v>55292</v>
+        <v>56177</v>
       </c>
       <c r="X15" s="19" t="n">
-        <v>74458</v>
+        <v>75343</v>
       </c>
       <c r="Y15" s="19" t="n">
-        <v>18585</v>
+        <v>19072</v>
       </c>
       <c r="Z15" s="19" t="n">
-        <v>153482</v>
+        <v>153465</v>
       </c>
       <c r="AA15" s="19" t="n">
-        <v>143783</v>
+        <v>143766</v>
       </c>
       <c r="AB15" s="19" t="n">
-        <v>-76438</v>
+        <v>-76442</v>
       </c>
       <c r="AC15" s="19" t="n">
-        <v>166895</v>
+        <v>166878</v>
       </c>
       <c r="AD15" s="19" t="n">
-        <v>176396</v>
+        <v>176379</v>
       </c>
       <c r="AE15" s="19" t="n">
-        <v>-65888</v>
+        <v>-65892</v>
       </c>
       <c r="AF15" s="19" t="n">
-        <v>199508</v>
+        <v>199491</v>
       </c>
       <c r="AG15" s="19" t="n">
-        <v>209009</v>
+        <v>208992</v>
       </c>
       <c r="AH15" s="19" t="n">
-        <v>-55337</v>
+        <v>-55341</v>
       </c>
       <c r="AI15" s="19" t="n">
-        <v>232120</v>
+        <v>232103</v>
       </c>
       <c r="AJ15" s="19" t="n">
-        <v>241622</v>
+        <v>241605</v>
       </c>
       <c r="AK15" s="19" t="n">
-        <v>-1757</v>
+        <v>-1761</v>
       </c>
     </row>
     <row r="16">
@@ -6164,112 +6164,112 @@
         </is>
       </c>
       <c r="B16" s="22" t="n">
-        <v>64859</v>
+        <v>64828</v>
       </c>
       <c r="C16" s="22" t="n">
-        <v>54663</v>
+        <v>54601</v>
       </c>
       <c r="D16" s="22" t="n">
-        <v>44790</v>
+        <v>44697</v>
       </c>
       <c r="E16" s="22" t="n">
-        <v>43448</v>
+        <v>43324</v>
       </c>
       <c r="F16" s="22" t="n">
-        <v>42366</v>
+        <v>42211</v>
       </c>
       <c r="G16" s="22" t="n">
-        <v>42269</v>
+        <v>42083</v>
       </c>
       <c r="H16" s="22" t="n">
-        <v>43961</v>
+        <v>43744</v>
       </c>
       <c r="I16" s="22" t="n">
-        <v>45912</v>
+        <v>45664</v>
       </c>
       <c r="J16" s="22" t="n">
-        <v>45417</v>
+        <v>45138</v>
       </c>
       <c r="K16" s="22" t="n">
-        <v>47628</v>
+        <v>47318</v>
       </c>
       <c r="L16" s="22" t="n">
-        <v>51998</v>
+        <v>51657</v>
       </c>
       <c r="M16" s="22" t="n">
-        <v>52233</v>
+        <v>51861</v>
       </c>
       <c r="N16" s="22" t="n">
-        <v>99829</v>
+        <v>100342</v>
       </c>
       <c r="O16" s="22" t="n">
-        <v>132385</v>
+        <v>133783</v>
       </c>
       <c r="P16" s="22" t="n">
-        <v>125829</v>
+        <v>127714</v>
       </c>
       <c r="Q16" s="22" t="n">
-        <v>163641</v>
+        <v>166411</v>
       </c>
       <c r="R16" s="22" t="n">
-        <v>213491</v>
+        <v>217146</v>
       </c>
       <c r="S16" s="22" t="n">
-        <v>211838</v>
+        <v>215980</v>
       </c>
       <c r="T16" s="22" t="n">
-        <v>256964</v>
+        <v>261991</v>
       </c>
       <c r="U16" s="22" t="n">
-        <v>305218</v>
+        <v>311130</v>
       </c>
       <c r="V16" s="22" t="n">
-        <v>303947</v>
+        <v>310346</v>
       </c>
       <c r="W16" s="22" t="n">
-        <v>359239</v>
+        <v>366523</v>
       </c>
       <c r="X16" s="22" t="n">
-        <v>433697</v>
+        <v>441866</v>
       </c>
       <c r="Y16" s="22" t="n">
-        <v>452282</v>
+        <v>460938</v>
       </c>
       <c r="Z16" s="22" t="n">
-        <v>605764</v>
+        <v>614403</v>
       </c>
       <c r="AA16" s="22" t="n">
-        <v>749547</v>
+        <v>758169</v>
       </c>
       <c r="AB16" s="22" t="n">
-        <v>673109</v>
+        <v>681727</v>
       </c>
       <c r="AC16" s="22" t="n">
-        <v>840004</v>
+        <v>848605</v>
       </c>
       <c r="AD16" s="22" t="n">
-        <v>1016400</v>
+        <v>1024984</v>
       </c>
       <c r="AE16" s="22" t="n">
-        <v>950512</v>
+        <v>959092</v>
       </c>
       <c r="AF16" s="22" t="n">
-        <v>1150020</v>
+        <v>1158583</v>
       </c>
       <c r="AG16" s="22" t="n">
-        <v>1359029</v>
+        <v>1367575</v>
       </c>
       <c r="AH16" s="22" t="n">
-        <v>1303692</v>
+        <v>1312234</v>
       </c>
       <c r="AI16" s="22" t="n">
-        <v>1535812</v>
+        <v>1544337</v>
       </c>
       <c r="AJ16" s="22" t="n">
-        <v>1777434</v>
+        <v>1785942</v>
       </c>
       <c r="AK16" s="22" t="n">
-        <v>1775677</v>
+        <v>1784181</v>
       </c>
     </row>
   </sheetData>
@@ -6368,7 +6368,7 @@
         <v>13</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>17590.75</v>
+        <v>17218.75</v>
       </c>
     </row>
     <row r="6">
@@ -6393,7 +6393,7 @@
         <v>8</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>33082</v>
+        <v>32865</v>
       </c>
     </row>
     <row r="7">
@@ -6418,7 +6418,7 @@
         <v>6</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>40093.472</v>
+        <v>39938.472</v>
       </c>
     </row>
     <row r="10">
@@ -6914,12 +6914,12 @@
       </c>
       <c r="B40" s="31" t="inlineStr">
         <is>
-          <t>4.25%</t>
+          <t>4.75%</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>corregido tras Miguel</t>
+          <t>Línea Emprendedores</t>
         </is>
       </c>
     </row>
@@ -6930,7 +6930,7 @@
         </is>
       </c>
       <c r="B41" s="31" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
@@ -6949,7 +6949,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>meses post-carencia</t>
+          <t>meses post-carencia (total 96)</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
         </is>
       </c>
       <c r="B43" s="31" t="n">
-        <v>1182</v>
+        <v>1199</v>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>

</xml_diff>